<commit_message>
update edit and delete user testcase
</commit_message>
<xml_diff>
--- a/src/test/resources/testdataCMS/CMS_DATA.xlsx
+++ b/src/test/resources/testdataCMS/CMS_DATA.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Learn\Automation\Automationorangehrmlive\src\test\resources\testdataCMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{624C048E-EC21-4B2F-9DAB-7148CA70721A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B48CF114-FCB1-4F7E-8CB9-E40268C4525A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{490F9023-B7EE-41AE-A955-F70AB61ADD8E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{490F9023-B7EE-41AE-A955-F70AB61ADD8E}"/>
   </bookViews>
   <sheets>
     <sheet name="AddUser" sheetId="1" r:id="rId1"/>
-    <sheet name="SearchUser" sheetId="2" r:id="rId2"/>
+    <sheet name="EditUser" sheetId="3" r:id="rId2"/>
+    <sheet name="SearchUser" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="26">
   <si>
     <t>employeeName</t>
   </si>
@@ -81,37 +82,40 @@
     <t>o</t>
   </si>
   <si>
-    <t>usertest0000001</t>
-  </si>
-  <si>
-    <t>usertest000002</t>
-  </si>
-  <si>
-    <t>usertest000003</t>
-  </si>
-  <si>
-    <t>usertest000004</t>
-  </si>
-  <si>
-    <t>usertest000005</t>
-  </si>
-  <si>
-    <t>usertest000006</t>
-  </si>
-  <si>
-    <t>usertest000007</t>
-  </si>
-  <si>
-    <t>usertest000008</t>
-  </si>
-  <si>
-    <t>usertest000009</t>
-  </si>
-  <si>
-    <t>usertest000010</t>
-  </si>
-  <si>
-    <t>usertest000011</t>
+    <t>usertes100000000000</t>
+  </si>
+  <si>
+    <t>usertest0000002</t>
+  </si>
+  <si>
+    <t>usertest0000003</t>
+  </si>
+  <si>
+    <t>usertest0000004</t>
+  </si>
+  <si>
+    <t>usertest0000005</t>
+  </si>
+  <si>
+    <t>usertest0000006</t>
+  </si>
+  <si>
+    <t>usertest0000007</t>
+  </si>
+  <si>
+    <t>usertest0000008</t>
+  </si>
+  <si>
+    <t>usertest0000009</t>
+  </si>
+  <si>
+    <t>usertest0000010</t>
+  </si>
+  <si>
+    <t>usertest0000011</t>
+  </si>
+  <si>
+    <t>usertest1000090000</t>
   </si>
 </sst>
 </file>
@@ -776,6 +780,157 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25CD02F7-8A0A-40F4-A5DB-27AD8B64D626}">
+  <dimension ref="A1:I15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+    </row>
+    <row r="3" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+    </row>
+    <row r="4" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+    </row>
+    <row r="5" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+    </row>
+    <row r="6" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+    </row>
+    <row r="7" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+    </row>
+    <row r="8" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+    </row>
+    <row r="9" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+    </row>
+    <row r="10" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+    </row>
+    <row r="11" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="A11" s="1"/>
+      <c r="B11" s="1"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+    </row>
+    <row r="12" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="A12" s="1"/>
+      <c r="B12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+    </row>
+    <row r="13" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+    </row>
+    <row r="14" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+    </row>
+    <row r="15" spans="1:9" ht="18" x14ac:dyDescent="0.35">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
+      <c r="F15" s="1"/>
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98F28A7C-CDA7-4270-8D9F-1501F73B5A22}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.35"/>

</xml_diff>